<commit_message>
updated gene summary doc and scripts
</commit_message>
<xml_diff>
--- a/bankole_2026/documentation/06_create_gene_summary_16mdg.xlsx
+++ b/bankole_2026/documentation/06_create_gene_summary_16mdg.xlsx
@@ -200,7 +200,7 @@
 - mono-exons. </t>
   </si>
   <si>
-    <t xml:space="preserve">aggregate_UJC_propReads_to_gene_summary.py</t>
+    <t xml:space="preserve">SCRIPTS/aggregate_UJC_propReads_to_gene_summary.py</t>
   </si>
   <si>
     <t xml:space="preserve">aggregate columns for most expressed UJC</t>
@@ -310,7 +310,7 @@
     <t xml:space="preserve">count flags for: annotation (annotated UJC, ISM, annotated ERP, novel ERP), and statistical tests results (sig female bias, sig male bias, no sig bias, statistically analyzable)</t>
   </si>
   <si>
-    <t xml:space="preserve">SCRIPTS/aggregate_UJC_propReads_to_gene_summary.py</t>
+    <t xml:space="preserve">SCRIPTS/aggregate_ERP_propReads_to_gene_summary.py</t>
   </si>
   <si>
     <t xml:space="preserve">For each gene, summarize the most expressed ERP_plus </t>
@@ -433,10 +433,11 @@
     <t xml:space="preserve">OUT/gene_summary_{species}.csv</t>
   </si>
   <si>
-    <t xml:space="preserve">Re-run steps 18-53 with </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCRIPTS/create_UJC_propReads_table.py
+    <t xml:space="preserve">Re-run steps 18-53 after filtering ujc to only those with at least 10 reads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCRIPTS/filter_datafile_jxnHash_threshold_min10reads.py
+SCRIPTS/create_UJC_propReads_table.py
 SCRIPTS/flag_annotation_status_and_bias_in_UJC_propReads_table.py
 SCRIPTS/aggregate_UJC_propReads_to_gene_summary.py
 SCRIPTS/create_ERP_propReads_table.py
@@ -448,7 +449,7 @@
 SCRIPTS/merge_genesetID_to_gene_summaries.py</t>
   </si>
   <si>
-    <t xml:space="preserve">submit_full_gene_summary_pipeline_min10reads.sh</t>
+    <t xml:space="preserve">SCRIPTS/submit_full_gene_summary_pipeline_min10reads.sh</t>
   </si>
   <si>
     <t xml:space="preserve">DATA/datafile_jxnHash_{genome}.csv
@@ -1380,8 +1381,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="236.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="1" t="s">
+    <row r="50" customFormat="false" ht="258.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
         <v>101</v>
       </c>
       <c r="C50" s="4" t="s">

</xml_diff>